<commit_message>
Update api register TestCase
</commit_message>
<xml_diff>
--- a/TestCases/API_Register_TestCase.xlsx
+++ b/TestCases/API_Register_TestCase.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DoAnNganh\SpringMediCareWeb-Selenium-Testing\TestCases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD786349-F660-463C-A542-9518E367E76A}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DFEA66D-22BF-48F6-9903-8391928F2661}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8940" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="89">
   <si>
     <t>TEST CASE</t>
   </si>
@@ -321,6 +321,9 @@
     <t>Bug: API chưa kiểm tra định dạng số điện thoại, và vẫn cho tạo tài khoản.</t>
   </si>
   <si>
+    <t>TCAPIRegisterRetest8</t>
+  </si>
+  <si>
     <t>TC-API-REGISTER-009</t>
   </si>
   <si>
@@ -344,6 +347,9 @@
   </si>
   <si>
     <t>Bug: API chưa kiểm tra định dạng email, và vẫn cho tạo tài khoản.</t>
+  </si>
+  <si>
+    <t>TCAPIRegisterRetest9</t>
   </si>
   <si>
     <t>TC-API-REGISTER-010</t>
@@ -370,15 +376,18 @@
   <si>
     <t>Bug: API chưa kiểm tra yêu cầu bảo mật của Password và vẫn cho phép tạo tài khoản với Password không hợp lệ.</t>
   </si>
+  <si>
+    <t>TCAPIRegisterRetest10</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="d\-m"/>
+    <numFmt numFmtId="164" formatCode="d\-m"/>
   </numFmts>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -426,6 +435,12 @@
       <sz val="11"/>
       <color rgb="FFFF0000"/>
       <name val="Tahoma"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
     </font>
   </fonts>
   <fills count="6">
@@ -590,7 +605,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
@@ -627,11 +642,14 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -897,16 +915,16 @@
     <col min="9" max="9" width="15.44140625" customWidth="1"/>
     <col min="10" max="10" width="21.33203125" customWidth="1"/>
     <col min="11" max="12" width="19.88671875" customWidth="1"/>
-    <col min="13" max="13" width="21.109375" customWidth="1"/>
+    <col min="13" max="13" width="26.33203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28"/>
+      <c r="B1" s="28"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
       <c r="E1" s="2"/>
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
@@ -933,9 +951,9 @@
     </row>
     <row r="2" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A2" s="2"/>
-      <c r="B2" s="26"/>
-      <c r="C2" s="26"/>
-      <c r="D2" s="26"/>
+      <c r="B2" s="27"/>
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
@@ -964,11 +982,11 @@
       <c r="A3" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="29" t="s">
+      <c r="B3" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="22"/>
-      <c r="D3" s="24"/>
+      <c r="C3" s="23"/>
+      <c r="D3" s="25"/>
       <c r="E3" s="2"/>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
@@ -997,11 +1015,11 @@
       <c r="A4" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="30" t="s">
+      <c r="B4" s="31" t="s">
         <v>22</v>
       </c>
-      <c r="C4" s="22"/>
-      <c r="D4" s="24"/>
+      <c r="C4" s="23"/>
+      <c r="D4" s="25"/>
       <c r="E4" s="2"/>
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
@@ -1030,11 +1048,11 @@
       <c r="A5" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="29" t="s">
+      <c r="B5" s="30" t="s">
         <v>23</v>
       </c>
-      <c r="C5" s="22"/>
-      <c r="D5" s="24"/>
+      <c r="C5" s="23"/>
+      <c r="D5" s="25"/>
       <c r="E5" s="2"/>
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
@@ -1163,39 +1181,39 @@
       <c r="AA8" s="3"/>
     </row>
     <row r="9" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A9" s="31" t="s">
+      <c r="A9" s="32" t="s">
         <v>9</v>
       </c>
-      <c r="B9" s="32" t="s">
+      <c r="B9" s="33" t="s">
         <v>10</v>
       </c>
-      <c r="C9" s="31" t="s">
+      <c r="C9" s="32" t="s">
         <v>11</v>
       </c>
-      <c r="D9" s="33" t="s">
+      <c r="D9" s="34" t="s">
         <v>12</v>
       </c>
-      <c r="E9" s="28"/>
-      <c r="F9" s="28"/>
-      <c r="G9" s="31" t="s">
+      <c r="E9" s="29"/>
+      <c r="F9" s="29"/>
+      <c r="G9" s="32" t="s">
         <v>13</v>
       </c>
-      <c r="H9" s="34" t="s">
+      <c r="H9" s="35" t="s">
         <v>14</v>
       </c>
-      <c r="I9" s="34" t="s">
+      <c r="I9" s="35" t="s">
         <v>15</v>
       </c>
-      <c r="J9" s="34" t="s">
+      <c r="J9" s="35" t="s">
         <v>16</v>
       </c>
-      <c r="K9" s="34" t="s">
+      <c r="K9" s="35" t="s">
         <v>17</v>
       </c>
-      <c r="L9" s="34" t="s">
+      <c r="L9" s="35" t="s">
         <v>18</v>
       </c>
-      <c r="M9" s="34" t="s">
+      <c r="M9" s="35" t="s">
         <v>19</v>
       </c>
       <c r="N9" s="3"/>
@@ -1214,19 +1232,19 @@
       <c r="AA9" s="3"/>
     </row>
     <row r="10" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A10" s="23"/>
-      <c r="B10" s="23"/>
-      <c r="C10" s="23"/>
-      <c r="D10" s="25"/>
-      <c r="E10" s="26"/>
-      <c r="F10" s="26"/>
-      <c r="G10" s="23"/>
-      <c r="H10" s="23"/>
-      <c r="I10" s="23"/>
-      <c r="J10" s="23"/>
-      <c r="K10" s="23"/>
-      <c r="L10" s="23"/>
-      <c r="M10" s="23"/>
+      <c r="A10" s="24"/>
+      <c r="B10" s="24"/>
+      <c r="C10" s="24"/>
+      <c r="D10" s="26"/>
+      <c r="E10" s="27"/>
+      <c r="F10" s="27"/>
+      <c r="G10" s="24"/>
+      <c r="H10" s="24"/>
+      <c r="I10" s="24"/>
+      <c r="J10" s="24"/>
+      <c r="K10" s="24"/>
+      <c r="L10" s="24"/>
+      <c r="M10" s="24"/>
       <c r="N10" s="3"/>
       <c r="O10" s="3"/>
       <c r="P10" s="3"/>
@@ -1248,14 +1266,14 @@
       <c r="C11" s="11"/>
       <c r="D11" s="11"/>
       <c r="E11" s="11"/>
-      <c r="F11" s="35"/>
-      <c r="G11" s="22"/>
-      <c r="H11" s="22"/>
-      <c r="I11" s="22"/>
-      <c r="J11" s="22"/>
-      <c r="K11" s="22"/>
-      <c r="L11" s="22"/>
-      <c r="M11" s="22"/>
+      <c r="F11" s="36"/>
+      <c r="G11" s="23"/>
+      <c r="H11" s="23"/>
+      <c r="I11" s="23"/>
+      <c r="J11" s="23"/>
+      <c r="K11" s="23"/>
+      <c r="L11" s="23"/>
+      <c r="M11" s="23"/>
       <c r="N11" s="3"/>
       <c r="O11" s="3"/>
       <c r="P11" s="3"/>
@@ -1272,21 +1290,21 @@
       <c r="AA11" s="3"/>
     </row>
     <row r="12" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A12" s="36" t="s">
+      <c r="A12" s="37" t="s">
         <v>20</v>
       </c>
-      <c r="B12" s="22"/>
-      <c r="C12" s="22"/>
-      <c r="D12" s="22"/>
-      <c r="E12" s="22"/>
-      <c r="F12" s="22"/>
-      <c r="G12" s="22"/>
-      <c r="H12" s="22"/>
-      <c r="I12" s="22"/>
-      <c r="J12" s="22"/>
-      <c r="K12" s="22"/>
-      <c r="L12" s="22"/>
-      <c r="M12" s="24"/>
+      <c r="B12" s="23"/>
+      <c r="C12" s="23"/>
+      <c r="D12" s="23"/>
+      <c r="E12" s="23"/>
+      <c r="F12" s="23"/>
+      <c r="G12" s="23"/>
+      <c r="H12" s="23"/>
+      <c r="I12" s="23"/>
+      <c r="J12" s="23"/>
+      <c r="K12" s="23"/>
+      <c r="L12" s="23"/>
+      <c r="M12" s="25"/>
       <c r="N12" s="3"/>
       <c r="O12" s="3"/>
       <c r="P12" s="3"/>
@@ -1312,11 +1330,11 @@
       <c r="C13" s="16" t="s">
         <v>26</v>
       </c>
-      <c r="D13" s="37" t="s">
+      <c r="D13" s="38" t="s">
         <v>27</v>
       </c>
-      <c r="E13" s="22"/>
-      <c r="F13" s="22"/>
+      <c r="E13" s="23"/>
+      <c r="F13" s="23"/>
       <c r="G13" s="17" t="s">
         <v>28</v>
       </c>
@@ -1348,21 +1366,21 @@
       <c r="AA13" s="3"/>
     </row>
     <row r="14" spans="1:27" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="36" t="s">
+      <c r="A14" s="37" t="s">
         <v>30</v>
       </c>
-      <c r="B14" s="22"/>
-      <c r="C14" s="22"/>
-      <c r="D14" s="22"/>
-      <c r="E14" s="22"/>
-      <c r="F14" s="22"/>
-      <c r="G14" s="22"/>
-      <c r="H14" s="22"/>
-      <c r="I14" s="22"/>
-      <c r="J14" s="22"/>
-      <c r="K14" s="22"/>
-      <c r="L14" s="22"/>
-      <c r="M14" s="24"/>
+      <c r="B14" s="23"/>
+      <c r="C14" s="23"/>
+      <c r="D14" s="23"/>
+      <c r="E14" s="23"/>
+      <c r="F14" s="23"/>
+      <c r="G14" s="23"/>
+      <c r="H14" s="23"/>
+      <c r="I14" s="23"/>
+      <c r="J14" s="23"/>
+      <c r="K14" s="23"/>
+      <c r="L14" s="23"/>
+      <c r="M14" s="25"/>
       <c r="N14" s="3"/>
       <c r="O14" s="3"/>
       <c r="P14" s="3"/>
@@ -1388,11 +1406,11 @@
       <c r="C15" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="D15" s="37" t="s">
+      <c r="D15" s="38" t="s">
         <v>33</v>
       </c>
-      <c r="E15" s="22"/>
-      <c r="F15" s="22"/>
+      <c r="E15" s="23"/>
+      <c r="F15" s="23"/>
       <c r="G15" s="17" t="s">
         <v>34</v>
       </c>
@@ -1406,7 +1424,7 @@
         <v>35</v>
       </c>
       <c r="K15" s="19"/>
-      <c r="L15" s="3"/>
+      <c r="L15" s="19"/>
       <c r="M15" s="20"/>
       <c r="N15" s="3"/>
       <c r="O15" s="3"/>
@@ -1433,11 +1451,11 @@
       <c r="C16" s="16" t="s">
         <v>38</v>
       </c>
-      <c r="D16" s="37" t="s">
+      <c r="D16" s="38" t="s">
         <v>39</v>
       </c>
-      <c r="E16" s="22"/>
-      <c r="F16" s="22"/>
+      <c r="E16" s="23"/>
+      <c r="F16" s="23"/>
       <c r="G16" s="17" t="s">
         <v>40</v>
       </c>
@@ -1469,21 +1487,21 @@
       <c r="AA16" s="3"/>
     </row>
     <row r="17" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A17" s="36" t="s">
+      <c r="A17" s="37" t="s">
         <v>42</v>
       </c>
-      <c r="B17" s="22"/>
-      <c r="C17" s="22"/>
-      <c r="D17" s="22"/>
-      <c r="E17" s="22"/>
-      <c r="F17" s="22"/>
-      <c r="G17" s="22"/>
-      <c r="H17" s="22"/>
-      <c r="I17" s="22"/>
-      <c r="J17" s="22"/>
-      <c r="K17" s="22"/>
-      <c r="L17" s="22"/>
-      <c r="M17" s="24"/>
+      <c r="B17" s="23"/>
+      <c r="C17" s="23"/>
+      <c r="D17" s="23"/>
+      <c r="E17" s="23"/>
+      <c r="F17" s="23"/>
+      <c r="G17" s="23"/>
+      <c r="H17" s="23"/>
+      <c r="I17" s="23"/>
+      <c r="J17" s="23"/>
+      <c r="K17" s="23"/>
+      <c r="L17" s="23"/>
+      <c r="M17" s="25"/>
       <c r="N17" s="3"/>
       <c r="O17" s="3"/>
       <c r="P17" s="3"/>
@@ -1509,11 +1527,11 @@
       <c r="C18" s="16" t="s">
         <v>45</v>
       </c>
-      <c r="D18" s="37" t="s">
+      <c r="D18" s="38" t="s">
         <v>46</v>
       </c>
-      <c r="E18" s="22"/>
-      <c r="F18" s="22"/>
+      <c r="E18" s="23"/>
+      <c r="F18" s="23"/>
       <c r="G18" s="17" t="s">
         <v>47</v>
       </c>
@@ -1554,11 +1572,11 @@
       <c r="C19" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="D19" s="37" t="s">
+      <c r="D19" s="38" t="s">
         <v>52</v>
       </c>
-      <c r="E19" s="22"/>
-      <c r="F19" s="22"/>
+      <c r="E19" s="23"/>
+      <c r="F19" s="23"/>
       <c r="G19" s="17" t="s">
         <v>53</v>
       </c>
@@ -1599,11 +1617,11 @@
       <c r="C20" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="D20" s="37" t="s">
+      <c r="D20" s="38" t="s">
         <v>58</v>
       </c>
-      <c r="E20" s="22"/>
-      <c r="F20" s="22"/>
+      <c r="E20" s="23"/>
+      <c r="F20" s="23"/>
       <c r="G20" s="17" t="s">
         <v>59</v>
       </c>
@@ -1644,11 +1662,11 @@
       <c r="C21" s="16" t="s">
         <v>63</v>
       </c>
-      <c r="D21" s="37" t="s">
+      <c r="D21" s="38" t="s">
         <v>64</v>
       </c>
-      <c r="E21" s="22"/>
-      <c r="F21" s="22"/>
+      <c r="E21" s="23"/>
+      <c r="F21" s="23"/>
       <c r="G21" s="17" t="s">
         <v>65</v>
       </c>
@@ -1680,21 +1698,21 @@
       <c r="AA21" s="3"/>
     </row>
     <row r="22" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A22" s="36" t="s">
+      <c r="A22" s="37" t="s">
         <v>67</v>
       </c>
-      <c r="B22" s="22"/>
-      <c r="C22" s="22"/>
-      <c r="D22" s="22"/>
-      <c r="E22" s="22"/>
-      <c r="F22" s="22"/>
-      <c r="G22" s="22"/>
-      <c r="H22" s="22"/>
-      <c r="I22" s="22"/>
-      <c r="J22" s="22"/>
-      <c r="K22" s="22"/>
-      <c r="L22" s="22"/>
-      <c r="M22" s="24"/>
+      <c r="B22" s="23"/>
+      <c r="C22" s="23"/>
+      <c r="D22" s="23"/>
+      <c r="E22" s="23"/>
+      <c r="F22" s="23"/>
+      <c r="G22" s="23"/>
+      <c r="H22" s="23"/>
+      <c r="I22" s="23"/>
+      <c r="J22" s="23"/>
+      <c r="K22" s="23"/>
+      <c r="L22" s="23"/>
+      <c r="M22" s="25"/>
       <c r="N22" s="3"/>
       <c r="O22" s="3"/>
       <c r="P22" s="3"/>
@@ -1720,11 +1738,11 @@
       <c r="C23" s="16" t="s">
         <v>70</v>
       </c>
-      <c r="D23" s="37" t="s">
+      <c r="D23" s="38" t="s">
         <v>71</v>
       </c>
-      <c r="E23" s="22"/>
-      <c r="F23" s="22"/>
+      <c r="E23" s="23"/>
+      <c r="F23" s="23"/>
       <c r="G23" s="17" t="s">
         <v>72</v>
       </c>
@@ -1737,9 +1755,15 @@
       <c r="J23" s="16" t="s">
         <v>73</v>
       </c>
-      <c r="K23" s="19"/>
-      <c r="L23" s="19"/>
-      <c r="M23" s="20"/>
+      <c r="K23" s="18">
+        <v>46228</v>
+      </c>
+      <c r="L23" s="14" t="s">
+        <v>5</v>
+      </c>
+      <c r="M23" s="21" t="s">
+        <v>74</v>
+      </c>
       <c r="N23" s="3"/>
       <c r="O23" s="3"/>
       <c r="P23" s="3"/>
@@ -1757,21 +1781,21 @@
     </row>
     <row r="24" spans="1:27" ht="102.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="14" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B24" s="15" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C24" s="16" t="s">
-        <v>76</v>
-      </c>
-      <c r="D24" s="37" t="s">
         <v>77</v>
       </c>
-      <c r="E24" s="22"/>
-      <c r="F24" s="22"/>
+      <c r="D24" s="38" t="s">
+        <v>78</v>
+      </c>
+      <c r="E24" s="23"/>
+      <c r="F24" s="23"/>
       <c r="G24" s="17" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="H24" s="18">
         <v>46227</v>
@@ -1780,11 +1804,17 @@
         <v>7</v>
       </c>
       <c r="J24" s="16" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
-      <c r="K24" s="19"/>
-      <c r="L24" s="19"/>
-      <c r="M24" s="20"/>
+      <c r="K24" s="18">
+        <v>46228</v>
+      </c>
+      <c r="L24" s="14" t="s">
+        <v>5</v>
+      </c>
+      <c r="M24" s="21" t="s">
+        <v>81</v>
+      </c>
       <c r="N24" s="3"/>
       <c r="O24" s="3"/>
       <c r="P24" s="3"/>
@@ -1802,21 +1832,21 @@
     </row>
     <row r="25" spans="1:27" ht="102.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="14" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B25" s="15" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="C25" s="16" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
-      <c r="D25" s="37" t="s">
-        <v>83</v>
+      <c r="D25" s="38" t="s">
+        <v>85</v>
       </c>
-      <c r="E25" s="22"/>
-      <c r="F25" s="22"/>
+      <c r="E25" s="23"/>
+      <c r="F25" s="23"/>
       <c r="G25" s="17" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="H25" s="18">
         <v>46227</v>
@@ -1825,11 +1855,17 @@
         <v>7</v>
       </c>
       <c r="J25" s="16" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
-      <c r="K25" s="19"/>
-      <c r="L25" s="19"/>
-      <c r="M25" s="20"/>
+      <c r="K25" s="18">
+        <v>46228</v>
+      </c>
+      <c r="L25" s="14" t="s">
+        <v>5</v>
+      </c>
+      <c r="M25" s="21" t="s">
+        <v>88</v>
+      </c>
       <c r="N25" s="3"/>
       <c r="O25" s="3"/>
       <c r="P25" s="3"/>
@@ -1934,7 +1970,7 @@
     </row>
     <row r="29" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A29" s="3"/>
-      <c r="B29" s="21"/>
+      <c r="B29" s="22"/>
       <c r="C29" s="3"/>
       <c r="D29" s="3"/>
       <c r="E29" s="3"/>
@@ -30180,36 +30216,36 @@
     </row>
   </sheetData>
   <mergeCells count="30">
+    <mergeCell ref="D21:F21"/>
+    <mergeCell ref="D23:F23"/>
+    <mergeCell ref="D24:F24"/>
+    <mergeCell ref="D25:F25"/>
+    <mergeCell ref="M9:M10"/>
     <mergeCell ref="F11:M11"/>
-    <mergeCell ref="D24:F24"/>
-    <mergeCell ref="D23:F23"/>
+    <mergeCell ref="A12:M12"/>
     <mergeCell ref="D13:F13"/>
+    <mergeCell ref="A14:M14"/>
     <mergeCell ref="D15:F15"/>
+    <mergeCell ref="A17:M17"/>
+    <mergeCell ref="A22:M22"/>
+    <mergeCell ref="L9:L10"/>
+    <mergeCell ref="D16:F16"/>
     <mergeCell ref="D18:F18"/>
-    <mergeCell ref="D16:F16"/>
-    <mergeCell ref="B5:D5"/>
-    <mergeCell ref="B4:D4"/>
-    <mergeCell ref="B3:D3"/>
-    <mergeCell ref="B1:D2"/>
-    <mergeCell ref="K9:K10"/>
-    <mergeCell ref="J9:J10"/>
-    <mergeCell ref="I9:I10"/>
-    <mergeCell ref="H9:H10"/>
-    <mergeCell ref="G9:G10"/>
-    <mergeCell ref="M9:M10"/>
-    <mergeCell ref="D9:F10"/>
-    <mergeCell ref="C9:C10"/>
-    <mergeCell ref="B9:B10"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="L9:L10"/>
-    <mergeCell ref="D21:F21"/>
-    <mergeCell ref="D25:F25"/>
-    <mergeCell ref="A17:M17"/>
-    <mergeCell ref="A12:M12"/>
-    <mergeCell ref="A22:M22"/>
     <mergeCell ref="D19:F19"/>
     <mergeCell ref="D20:F20"/>
-    <mergeCell ref="A14:M14"/>
+    <mergeCell ref="G9:G10"/>
+    <mergeCell ref="H9:H10"/>
+    <mergeCell ref="I9:I10"/>
+    <mergeCell ref="J9:J10"/>
+    <mergeCell ref="K9:K10"/>
+    <mergeCell ref="B1:D2"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="D9:F10"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="G13" r:id="rId1" xr:uid="{00000000-0004-0000-0600-000000000000}"/>
@@ -30220,8 +30256,11 @@
     <hyperlink ref="G20" r:id="rId6" xr:uid="{00000000-0004-0000-0600-000005000000}"/>
     <hyperlink ref="G21" r:id="rId7" xr:uid="{00000000-0004-0000-0600-000006000000}"/>
     <hyperlink ref="G23" r:id="rId8" xr:uid="{00000000-0004-0000-0600-000007000000}"/>
-    <hyperlink ref="G24" r:id="rId9" xr:uid="{00000000-0004-0000-0600-000008000000}"/>
-    <hyperlink ref="G25" r:id="rId10" xr:uid="{00000000-0004-0000-0600-000009000000}"/>
+    <hyperlink ref="M23" r:id="rId9" xr:uid="{00000000-0004-0000-0600-000008000000}"/>
+    <hyperlink ref="G24" r:id="rId10" xr:uid="{00000000-0004-0000-0600-000009000000}"/>
+    <hyperlink ref="M24" r:id="rId11" xr:uid="{00000000-0004-0000-0600-00000A000000}"/>
+    <hyperlink ref="G25" r:id="rId12" xr:uid="{00000000-0004-0000-0600-00000B000000}"/>
+    <hyperlink ref="M25" r:id="rId13" xr:uid="{00000000-0004-0000-0600-00000C000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>